<commit_message>
v0.0.4 prep commit. Logging cleanliness. Logo. Tested Compilation process. Pending fix for filelock not being installed from wheel
</commit_message>
<xml_diff>
--- a/xlpro_examples/xlpro-ex01-basics.xlsx
+++ b/xlpro_examples/xlpro-ex01-basics.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Daniel Evans\projects\xlpro\xlpro_examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{531CEBA7-3C3E-4DC3-8170-8FD369D520D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F6F31E0-BF26-4C78-806F-2FF0049A3227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21000" xr2:uid="{6E9394D3-1908-4984-B373-92B4E72AC2C6}"/>
   </bookViews>
@@ -24,6 +24,7 @@
     <definedName name="args_custom_adder_always_vector">{"vector";"constant"}</definedName>
     <definedName name="args_custom_adder_matrix">{"matrix";"constant"}</definedName>
     <definedName name="args_deepcpy">"val"</definedName>
+    <definedName name="args_get_banana_price">""</definedName>
     <definedName name="args_hello">"name"</definedName>
     <definedName name="args_pyadd">{"val";"rhs"}</definedName>
     <definedName name="args_pydiv">{"val";"rhs"}</definedName>
@@ -56,6 +57,7 @@
     <definedName name="fname_custom_adder_always_vector">"custom_adder_always_vector"</definedName>
     <definedName name="fname_custom_adder_matrix">"custom_adder_matrix"</definedName>
     <definedName name="fname_deepcpy">"deepcpy"</definedName>
+    <definedName name="fname_get_banana_price">"get_banana_price"</definedName>
     <definedName name="fname_hello">"hello"</definedName>
     <definedName name="fname_pyadd">"pyadd"</definedName>
     <definedName name="fname_pydiv">"pydiv"</definedName>
@@ -104,7 +106,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -368,8 +370,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="5734706" y="5543216"/>
-          <a:ext cx="3237615" cy="2293684"/>
+          <a:off x="5669872" y="5543216"/>
+          <a:ext cx="3201596" cy="2293684"/>
           <a:chOff x="5594578" y="4920377"/>
           <a:chExt cx="3224992" cy="2293684"/>
         </a:xfrm>
@@ -804,10 +806,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="93" name="figure1">
+        <xdr:cNvPr id="9" name="figure1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{31CA42ED-B6DE-F255-3905-40DD761673CA}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A1010D3C-5D11-8E7C-ADD8-B98DCE4C0FC6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2101,7 +2103,7 @@
         <v>3</v>
       </c>
       <c r="C47" s="7">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D47" s="7">
         <v>13</v>
@@ -2112,13 +2114,13 @@
       <c r="F47" s="3"/>
       <c r="G47" s="8" t="str" cm="1">
         <f t="array" ref="G47">custom_adder_matrix(C47:E48,$C$45)</f>
-        <v>PyObj&lt;Sheet1$G$4732f73c31bd634fbc5bf0cf095ad3d1105b6b0a1ba091c758fb5827ea312eef1d&gt;</v>
+        <v>PyObj&lt;Sheet1$G$47faa0e9486d6d0f4b61c5f1703b7755d5c27e4f3759a412d3f86649185c2e27dd&gt;</v>
       </c>
       <c r="I47" s="3"/>
       <c r="J47" s="3"/>
       <c r="K47" s="8" cm="1">
         <f t="array" ref="K47:M48">show(G47)</f>
-        <v>11.412000000000001</v>
+        <v>22.411999999999999</v>
       </c>
       <c r="L47" s="8">
         <v>22.411999999999999</v>

</xml_diff>